<commit_message>
min value updated to 0.1
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/agent/STF agent - One valid row.xlsx
+++ b/src/test/resources/testData/agent/STF agent - One valid row.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/karthik.jaladurgam/Desktop/STOS/Test data/Agent/Automation/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/karthik.jaladurgam/workspace/securities-transfer-charge-submissions-ui-tests/src/test/resources/testData/agent/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66EF2AE1-E910-5640-8EDB-776DB177ED98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{975BAC64-E3DC-7742-B108-1269410BF6B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1141,7 +1141,7 @@
         <v>400</v>
       </c>
       <c r="AC4" s="13">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="AD4" s="5"/>
       <c r="AE4" s="5"/>

</xml_diff>